<commit_message>
Done. The two visible references to "SmartBooks" inside the spreadsheet (the title on the Summary tab and the pitch one-liner) are now **"Business Software"**. Generator script updated too, so any future rebuild keeps the change.
The filename `SmartBooks_Cost_Model.xlsx` is unchanged — say the word if you'd like me to rename that too.

**[SmartBooks_Cost_Model.xlsx](https://aifinance-hub-6.preview.emergentagent.com/downloads/SmartBooks_Cost_Model.xlsx)**
</commit_message>
<xml_diff>
--- a/frontend/public/downloads/SmartBooks_Cost_Model.xlsx
+++ b/frontend/public/downloads/SmartBooks_Cost_Model.xlsx
@@ -599,7 +599,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SmartBooks — Tech-Only Cost Model (v5, Feb 2026)</t>
+          <t>Business Software — Tech-Only Cost Model (v5, Feb 2026)</t>
         </is>
       </c>
     </row>
@@ -610,6 +610,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -755,6 +756,7 @@
       </c>
       <c r="F10" s="9" t="inlineStr"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -836,6 +838,8 @@
       <c r="E16" s="5" t="inlineStr"/>
       <c r="F16" s="5" t="inlineStr"/>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -961,6 +965,8 @@
       </c>
       <c r="F25" s="5" t="inlineStr"/>
     </row>
+    <row r="26"/>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -971,7 +977,7 @@
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>At 1,500 paid users on a blended $71 ARPU, SmartBooks runs ~$11k/mo of pure tech cost against ~$106k MRR — 90% gross margin on the infra layer. Today's pre-revenue burn is ~$15.5k/mo of which $12k is temporary build velocity that tapers by month 6.</t>
+          <t>At 1,500 paid users on a blended $71 ARPU, Business Software runs ~$11k/mo of pure tech cost against ~$106k MRR — 90% gross margin on the infra layer. Today's pre-revenue burn is ~$15.5k/mo of which $12k is temporary build velocity that tapers by month 6.</t>
         </is>
       </c>
     </row>
@@ -1021,6 +1027,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1118,6 +1125,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -1169,6 +1177,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -1334,6 +1343,8 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -1495,6 +1506,8 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
@@ -1691,6 +1704,8 @@
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr"/>
     </row>
+    <row r="47"/>
+    <row r="48"/>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
@@ -1807,6 +1822,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2069,6 +2085,7 @@
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="14" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -2171,6 +2188,7 @@
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="16" t="n"/>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -2333,6 +2351,7 @@
       <c r="C34" s="18" t="n"/>
       <c r="D34" s="18" t="n"/>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
@@ -2346,6 +2365,7 @@
       <c r="C36" s="14" t="n"/>
       <c r="D36" s="14" t="n"/>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
@@ -2455,6 +2475,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2622,6 +2643,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -3012,6 +3035,7 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
@@ -3082,6 +3106,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
         <is>
@@ -3136,6 +3161,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="29" t="inlineStr">
         <is>
@@ -3147,6 +3173,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
@@ -3338,6 +3365,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3569,6 +3597,8 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -3960,6 +3990,8 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
@@ -4209,6 +4241,8 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
@@ -4310,6 +4344,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -4922,6 +4957,7 @@
         <v>150</v>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
@@ -5024,6 +5060,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5289,6 +5326,8 @@
         <v>0.003</v>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -5437,6 +5476,8 @@
         <v>70</v>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
@@ -5627,6 +5668,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -6359,6 +6401,7 @@
         <v>240</v>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
@@ -6391,6 +6434,7 @@
         <v/>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="31" t="inlineStr">
         <is>
@@ -6466,6 +6510,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -6687,6 +6732,8 @@
       <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -6908,6 +6955,8 @@
       <c r="H23" s="5" t="inlineStr"/>
       <c r="I23" s="5" t="inlineStr"/>
     </row>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -7165,6 +7214,8 @@
         <v>2651000.000000001</v>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
@@ -7341,6 +7392,8 @@
       <c r="H44" s="5" t="inlineStr"/>
       <c r="I44" s="5" t="inlineStr"/>
     </row>
+    <row r="45"/>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
@@ -7495,6 +7548,8 @@
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr"/>
     </row>
+    <row r="53"/>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
@@ -7549,6 +7604,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7686,6 +7742,8 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -7916,6 +7974,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -8146,6 +8206,8 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
@@ -8379,6 +8441,8 @@
         <v>0.2551935788479697</v>
       </c>
     </row>
+    <row r="40"/>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>

</xml_diff>